<commit_message>
Variable type and memory parsimony updates
</commit_message>
<xml_diff>
--- a/project1/deliverables/data.xlsx
+++ b/project1/deliverables/data.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I430"/>
+  <dimension ref="A1:H430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -446,10 +446,9 @@
     <col width="67" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="19" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="68" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="68" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -696,7 +695,6 @@
       <c r="E12" s="1" t="n"/>
       <c r="F12" s="1" t="n"/>
       <c r="G12" s="1" t="n"/>
-      <c r="H12" s="1" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -726,15 +724,10 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Audio URI</t>
+          <t>Audio Checksum</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Audio Checksum</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Ingest Status</t>
         </is>
@@ -760,15 +753,10 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/04/4817.flac</t>
+          <t>0xBD675D48363DAAFDCEF52552ABD98D2302AE34C58A6AEBE32A13ABF4A14ED8B4</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>0xBD675D48363DAAFDCEF52552ABD98D2302AE34C58A6AEBE32A13ABF4A14ED8B4</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -794,15 +782,10 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/04/4818.flac</t>
+          <t>0x5983C502A7DC729DE1309DB3472114C928E90E2E71279EDB90A32798A3091884</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>0x5983C502A7DC729DE1309DB3472114C928E90E2E71279EDB90A32798A3091884</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -828,15 +811,10 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/02/4819.flac</t>
+          <t>0x9E0DADD51ACFB2BFCFDCE10D63542D6F6C8B83DFCCF5FB602CA46A54419090E0</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>0x9E0DADD51ACFB2BFCFDCE10D63542D6F6C8B83DFCCF5FB602CA46A54419090E0</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -862,15 +840,10 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/03/4820.flac</t>
+          <t>0x957C70149E1299D5F80FD0662D0FE441DEA2F2CF3A794F01723649800FF79578</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>0x957C70149E1299D5F80FD0662D0FE441DEA2F2CF3A794F01723649800FF79578</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -896,15 +869,10 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/03/4821.flac</t>
+          <t>0x2555040D4C50FDD2636C8FD581A3D89945DDBF766A1CFD23D1C4E4A6A3F4D4B8</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>0x2555040D4C50FDD2636C8FD581A3D89945DDBF766A1CFD23D1C4E4A6A3F4D4B8</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -930,15 +898,10 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/05/4822.flac</t>
+          <t>0xD276CB55DFBBAC0965C4BBE6FD22644E4204016CB93E774BCA56AF5DCFA61122</t>
         </is>
       </c>
       <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>0xD276CB55DFBBAC0965C4BBE6FD22644E4204016CB93E774BCA56AF5DCFA61122</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -964,15 +927,10 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/03/4823.flac</t>
+          <t>0xC06597DE02EBD6D6AC031CB28019E44E4E5C12CDE2C78769A224FBFD1501C1C0</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>0xC06597DE02EBD6D6AC031CB28019E44E4E5C12CDE2C78769A224FBFD1501C1C0</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -998,15 +956,10 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/05/4824.flac</t>
+          <t>0x0648B585C6E9879E6C9673AB19090CBDF80BE8028F36134983CD256603CA5FE1</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>0x0648B585C6E9879E6C9673AB19090CBDF80BE8028F36134983CD256603CA5FE1</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -1032,15 +985,10 @@
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/05/4825.flac</t>
+          <t>0xD13AB16A153AC5FD800A4A10B9C8D8965BC0E1C4DB91898EFDE205E2ECD49DDC</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>0xD13AB16A153AC5FD800A4A10B9C8D8965BC0E1C4DB91898EFDE205E2ECD49DDC</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -1066,15 +1014,10 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/06/4826.flac</t>
+          <t>0x84385F82766187C8310ADBC23C28FB91EC47264C49137ABB45819B77E5708698</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>0x84385F82766187C8310ADBC23C28FB91EC47264C49137ABB45819B77E5708698</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -1100,15 +1043,10 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/05/4827.flac</t>
+          <t>0xB20784242490346AE77A68D7538C9AEC54488DF7B8F373C4FAC8835C0FA878CD</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>0xB20784242490346AE77A68D7538C9AEC54488DF7B8F373C4FAC8835C0FA878CD</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -1134,15 +1072,10 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/07/4828.flac</t>
+          <t>0x8B03F255CE532E687B4D146692737F2135AEF1B2AABB7C8DBE3AF0349EFB4B77</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>0x8B03F255CE532E687B4D146692737F2135AEF1B2AABB7C8DBE3AF0349EFB4B77</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -1168,15 +1101,10 @@
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/06/4829.flac</t>
+          <t>0x4F9FF37AD95773DCD6CADECE159F4EB187B0110E3B7F056B01B9CCC94773AE90</t>
         </is>
       </c>
       <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>0x4F9FF37AD95773DCD6CADECE159F4EB187B0110E3B7F056B01B9CCC94773AE90</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>scored</t>
         </is>
@@ -1202,15 +1130,10 @@
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/09/4830.flac</t>
+          <t>0x7D19F53A1DAF42AD0CF5F5891779E666A137A68AD890F95356FDDBA2F8E39417</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
-        <is>
-          <t>0x7D19F53A1DAF42AD0CF5F5891779E666A137A68AD890F95356FDDBA2F8E39417</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>awaiting scoring</t>
         </is>
@@ -1236,15 +1159,10 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>audio/2026/09/4831.flac</t>
+          <t>0x9261DDFAF151557C46D8A3DFB862D09D196E0BC6A34CFCEA97B5041AAE9D96F7</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>0x9261DDFAF151557C46D8A3DFB862D09D196E0BC6A34CFCEA97B5041AAE9D96F7</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>rejected</t>
         </is>
@@ -2127,7 +2045,6 @@
       <c r="F73" s="1" t="n"/>
       <c r="G73" s="1" t="n"/>
       <c r="H73" s="1" t="n"/>
-      <c r="I73" s="1" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -2166,11 +2083,6 @@
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
-        <is>
-          <t>Embedding Reference</t>
-        </is>
-      </c>
-      <c r="I74" s="2" t="inlineStr">
         <is>
           <t>Scored On</t>
         </is>
@@ -2198,12 +2110,7 @@
       <c r="G75" s="6" t="n">
         <v>0.0243</v>
       </c>
-      <c r="H75" s="3" t="inlineStr">
-        <is>
-          <t>beardown/4817</t>
-        </is>
-      </c>
-      <c r="I75" s="8" t="n">
+      <c r="H75" s="8" t="n">
         <v>46096.8971875</v>
       </c>
     </row>
@@ -2229,12 +2136,7 @@
       <c r="G76" s="6" t="n">
         <v>0.0058</v>
       </c>
-      <c r="H76" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm_cfg12/4817</t>
-        </is>
-      </c>
-      <c r="I76" s="8" t="n">
+      <c r="H76" s="8" t="n">
         <v>46115.58488425926</v>
       </c>
     </row>
@@ -2260,12 +2162,7 @@
       <c r="G77" s="6" t="n">
         <v>0.0289</v>
       </c>
-      <c r="H77" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm/4817</t>
-        </is>
-      </c>
-      <c r="I77" s="8" t="n">
+      <c r="H77" s="8" t="n">
         <v>46117.67543981481</v>
       </c>
     </row>
@@ -2291,12 +2188,7 @@
       <c r="G78" s="6" t="n">
         <v>0.0051</v>
       </c>
-      <c r="H78" s="3" t="inlineStr">
-        <is>
-          <t>beardown_3sec/4817</t>
-        </is>
-      </c>
-      <c r="I78" s="8" t="n">
+      <c r="H78" s="8" t="n">
         <v>46204.38532407407</v>
       </c>
     </row>
@@ -2322,12 +2214,7 @@
       <c r="G79" s="6" t="n">
         <v>0.0111</v>
       </c>
-      <c r="H79" s="3" t="inlineStr">
-        <is>
-          <t>beardown/4818</t>
-        </is>
-      </c>
-      <c r="I79" s="8" t="n">
+      <c r="H79" s="8" t="n">
         <v>46096.78737268518</v>
       </c>
     </row>
@@ -2353,12 +2240,7 @@
       <c r="G80" s="6" t="n">
         <v>0.0109</v>
       </c>
-      <c r="H80" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm/4818</t>
-        </is>
-      </c>
-      <c r="I80" s="8" t="n">
+      <c r="H80" s="8" t="n">
         <v>46138.44931712963</v>
       </c>
     </row>
@@ -2384,12 +2266,7 @@
       <c r="G81" s="6" t="n">
         <v>0.0105</v>
       </c>
-      <c r="H81" s="3" t="inlineStr">
-        <is>
-          <t>beardown/4819</t>
-        </is>
-      </c>
-      <c r="I81" s="8" t="n">
+      <c r="H81" s="8" t="n">
         <v>46043.01435185185</v>
       </c>
     </row>
@@ -2415,12 +2292,7 @@
       <c r="G82" s="6" t="n">
         <v>0.0233</v>
       </c>
-      <c r="H82" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm_cfg12/4819</t>
-        </is>
-      </c>
-      <c r="I82" s="8" t="n">
+      <c r="H82" s="8" t="n">
         <v>46082.44153935185</v>
       </c>
     </row>
@@ -2446,12 +2318,7 @@
       <c r="G83" s="6" t="n">
         <v>0.0057</v>
       </c>
-      <c r="H83" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm_cfg12/4820</t>
-        </is>
-      </c>
-      <c r="I83" s="8" t="n">
+      <c r="H83" s="8" t="n">
         <v>46070.78189814815</v>
       </c>
     </row>
@@ -2477,12 +2344,7 @@
       <c r="G84" s="6" t="n">
         <v>0.0256</v>
       </c>
-      <c r="H84" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm/4820</t>
-        </is>
-      </c>
-      <c r="I84" s="8" t="n">
+      <c r="H84" s="8" t="n">
         <v>46112.82530092593</v>
       </c>
     </row>
@@ -2508,12 +2370,7 @@
       <c r="G85" s="6" t="n">
         <v>0.0081</v>
       </c>
-      <c r="H85" s="3" t="inlineStr">
-        <is>
-          <t>beardown/4821</t>
-        </is>
-      </c>
-      <c r="I85" s="8" t="n">
+      <c r="H85" s="8" t="n">
         <v>46057.78736111111</v>
       </c>
     </row>
@@ -2539,12 +2396,7 @@
       <c r="G86" s="6" t="n">
         <v>0.0288</v>
       </c>
-      <c r="H86" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm_cfg12/4821</t>
-        </is>
-      </c>
-      <c r="I86" s="8" t="n">
+      <c r="H86" s="8" t="n">
         <v>46087.69145833333</v>
       </c>
     </row>
@@ -2570,12 +2422,7 @@
       <c r="G87" s="6" t="n">
         <v>0.0276</v>
       </c>
-      <c r="H87" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm/4822</t>
-        </is>
-      </c>
-      <c r="I87" s="8" t="n">
+      <c r="H87" s="8" t="n">
         <v>46105.44788194444</v>
       </c>
     </row>
@@ -2601,12 +2448,7 @@
       <c r="G88" s="6" t="n">
         <v>0.0121</v>
       </c>
-      <c r="H88" s="3" t="inlineStr">
-        <is>
-          <t>beardown_3sec/4822</t>
-        </is>
-      </c>
-      <c r="I88" s="8" t="n">
+      <c r="H88" s="8" t="n">
         <v>46199.24421296296</v>
       </c>
     </row>
@@ -2632,12 +2474,7 @@
       <c r="G89" s="6" t="n">
         <v>0.0128</v>
       </c>
-      <c r="H89" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm_cfg12/4823</t>
-        </is>
-      </c>
-      <c r="I89" s="8" t="n">
+      <c r="H89" s="8" t="n">
         <v>46081.96149305555</v>
       </c>
     </row>
@@ -2663,12 +2500,7 @@
       <c r="G90" s="6" t="n">
         <v>0.0179</v>
       </c>
-      <c r="H90" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm/4823</t>
-        </is>
-      </c>
-      <c r="I90" s="8" t="n">
+      <c r="H90" s="8" t="n">
         <v>46105.66568287037</v>
       </c>
     </row>
@@ -2692,12 +2524,7 @@
       <c r="G91" s="6" t="n">
         <v>0.0089</v>
       </c>
-      <c r="H91" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm/4824</t>
-        </is>
-      </c>
-      <c r="I91" s="8" t="n">
+      <c r="H91" s="8" t="n">
         <v>46105.72203703703</v>
       </c>
     </row>
@@ -2723,12 +2550,7 @@
       <c r="G92" s="6" t="n">
         <v>0.0273</v>
       </c>
-      <c r="H92" s="3" t="inlineStr">
-        <is>
-          <t>beardown/4825</t>
-        </is>
-      </c>
-      <c r="I92" s="8" t="n">
+      <c r="H92" s="8" t="n">
         <v>46124.13363425926</v>
       </c>
     </row>
@@ -2754,12 +2576,7 @@
       <c r="G93" s="6" t="n">
         <v>0.0246</v>
       </c>
-      <c r="H93" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm/4825</t>
-        </is>
-      </c>
-      <c r="I93" s="8" t="n">
+      <c r="H93" s="8" t="n">
         <v>46149.92591435185</v>
       </c>
     </row>
@@ -2785,12 +2602,7 @@
       <c r="G94" s="6" t="n">
         <v>0.018</v>
       </c>
-      <c r="H94" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm/4826</t>
-        </is>
-      </c>
-      <c r="I94" s="8" t="n">
+      <c r="H94" s="8" t="n">
         <v>46124.48695601852</v>
       </c>
     </row>
@@ -2816,12 +2628,7 @@
       <c r="G95" s="6" t="n">
         <v>0.0193</v>
       </c>
-      <c r="H95" s="3" t="inlineStr">
-        <is>
-          <t>beardown_3sec/4826</t>
-        </is>
-      </c>
-      <c r="I95" s="8" t="n">
+      <c r="H95" s="8" t="n">
         <v>46206.7353125</v>
       </c>
     </row>
@@ -2847,12 +2654,7 @@
       <c r="G96" s="6" t="n">
         <v>0.0117</v>
       </c>
-      <c r="H96" s="3" t="inlineStr">
-        <is>
-          <t>beardown/4827</t>
-        </is>
-      </c>
-      <c r="I96" s="8" t="n">
+      <c r="H96" s="8" t="n">
         <v>46145.62171296297</v>
       </c>
     </row>
@@ -2878,12 +2680,7 @@
       <c r="G97" s="6" t="n">
         <v>0.0072</v>
       </c>
-      <c r="H97" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm/4827</t>
-        </is>
-      </c>
-      <c r="I97" s="8" t="n">
+      <c r="H97" s="8" t="n">
         <v>46173.14605324074</v>
       </c>
     </row>
@@ -2909,12 +2706,7 @@
       <c r="G98" s="6" t="n">
         <v>0.0054</v>
       </c>
-      <c r="H98" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm_cfg12/4828</t>
-        </is>
-      </c>
-      <c r="I98" s="8" t="n">
+      <c r="H98" s="8" t="n">
         <v>46145.58298611111</v>
       </c>
     </row>
@@ -2940,12 +2732,7 @@
       <c r="G99" s="6" t="n">
         <v>0.0246</v>
       </c>
-      <c r="H99" s="3" t="inlineStr">
-        <is>
-          <t>beardown_3sec/4828</t>
-        </is>
-      </c>
-      <c r="I99" s="8" t="n">
+      <c r="H99" s="8" t="n">
         <v>46218.42115740741</v>
       </c>
     </row>
@@ -2971,12 +2758,7 @@
       <c r="G100" s="6" t="n">
         <v>0.0265</v>
       </c>
-      <c r="H100" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm_cfg12/4829</t>
-        </is>
-      </c>
-      <c r="I100" s="8" t="n">
+      <c r="H100" s="8" t="n">
         <v>46162.66717592593</v>
       </c>
     </row>
@@ -3002,12 +2784,7 @@
       <c r="G101" s="6" t="n">
         <v>0.0036</v>
       </c>
-      <c r="H101" s="3" t="inlineStr">
-        <is>
-          <t>beardown_rrm/4829</t>
-        </is>
-      </c>
-      <c r="I101" s="8" t="n">
+      <c r="H101" s="8" t="n">
         <v>46182.7936574074</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Variable type and memory parsimony updates - mk2
</commit_message>
<xml_diff>
--- a/project1/deliverables/data.xlsx
+++ b/project1/deliverables/data.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="167" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="168" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,12 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <i val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -61,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="centerContinuous"/>
@@ -72,6 +78,7 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -147,6 +154,46 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>CROSSFADE</author>
+  </authors>
+  <commentList>
+    <comment ref="C74" authorId="0" shapeId="0">
+      <text>
+        <t>Derived: the genre with the highest Probability among this score's ten Genre Probability rows.</t>
+      </text>
+    </comment>
+    <comment ref="D74" authorId="0" shapeId="0">
+      <text>
+        <t>Derived: the largest of this score's ten Genre Probability values.</t>
+      </text>
+    </comment>
+    <comment ref="E74" authorId="0" shapeId="0">
+      <text>
+        <t>Derived: Shannon entropy of this score's ten probabilities divided by log(10), so 0 to 1.</t>
+      </text>
+    </comment>
+    <comment ref="F74" authorId="0" shapeId="0">
+      <text>
+        <t>Derived: mean Jensen-Shannon divergence (base 2) from the other models' distributions for the same track. Empty while only one model has scored it.</t>
+      </text>
+    </comment>
+    <comment ref="F399" authorId="0" shapeId="0">
+      <text>
+        <t>Derived: 1 exactly when Seconds Played equals the track's Duration.</t>
+      </text>
+    </comment>
+    <comment ref="H399" authorId="0" shapeId="0">
+      <text>
+        <t>Snapshot: the artist's Payout Rate at play time when Seconds Played is at least 30, otherwise 0. Copied, not looked up, so a later rate change never rewrites the ledger.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2057,22 +2104,22 @@
           <t>Model ID</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
+      <c r="C74" s="8" t="inlineStr">
         <is>
           <t>Genre ID</t>
         </is>
       </c>
-      <c r="D74" s="2" t="inlineStr">
+      <c r="D74" s="8" t="inlineStr">
         <is>
           <t>Top Probability</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
+      <c r="E74" s="8" t="inlineStr">
         <is>
           <t>Posterior Entropy</t>
         </is>
       </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="F74" s="8" t="inlineStr">
         <is>
           <t>Model Divergence</t>
         </is>
@@ -2110,7 +2157,7 @@
       <c r="G75" s="6" t="n">
         <v>0.0243</v>
       </c>
-      <c r="H75" s="8" t="n">
+      <c r="H75" s="9" t="n">
         <v>46096.8971875</v>
       </c>
     </row>
@@ -2136,7 +2183,7 @@
       <c r="G76" s="6" t="n">
         <v>0.0058</v>
       </c>
-      <c r="H76" s="8" t="n">
+      <c r="H76" s="9" t="n">
         <v>46115.58488425926</v>
       </c>
     </row>
@@ -2162,7 +2209,7 @@
       <c r="G77" s="6" t="n">
         <v>0.0289</v>
       </c>
-      <c r="H77" s="8" t="n">
+      <c r="H77" s="9" t="n">
         <v>46117.67543981481</v>
       </c>
     </row>
@@ -2188,7 +2235,7 @@
       <c r="G78" s="6" t="n">
         <v>0.0051</v>
       </c>
-      <c r="H78" s="8" t="n">
+      <c r="H78" s="9" t="n">
         <v>46204.38532407407</v>
       </c>
     </row>
@@ -2214,7 +2261,7 @@
       <c r="G79" s="6" t="n">
         <v>0.0111</v>
       </c>
-      <c r="H79" s="8" t="n">
+      <c r="H79" s="9" t="n">
         <v>46096.78737268518</v>
       </c>
     </row>
@@ -2240,7 +2287,7 @@
       <c r="G80" s="6" t="n">
         <v>0.0109</v>
       </c>
-      <c r="H80" s="8" t="n">
+      <c r="H80" s="9" t="n">
         <v>46138.44931712963</v>
       </c>
     </row>
@@ -2266,7 +2313,7 @@
       <c r="G81" s="6" t="n">
         <v>0.0105</v>
       </c>
-      <c r="H81" s="8" t="n">
+      <c r="H81" s="9" t="n">
         <v>46043.01435185185</v>
       </c>
     </row>
@@ -2292,7 +2339,7 @@
       <c r="G82" s="6" t="n">
         <v>0.0233</v>
       </c>
-      <c r="H82" s="8" t="n">
+      <c r="H82" s="9" t="n">
         <v>46082.44153935185</v>
       </c>
     </row>
@@ -2318,7 +2365,7 @@
       <c r="G83" s="6" t="n">
         <v>0.0057</v>
       </c>
-      <c r="H83" s="8" t="n">
+      <c r="H83" s="9" t="n">
         <v>46070.78189814815</v>
       </c>
     </row>
@@ -2344,7 +2391,7 @@
       <c r="G84" s="6" t="n">
         <v>0.0256</v>
       </c>
-      <c r="H84" s="8" t="n">
+      <c r="H84" s="9" t="n">
         <v>46112.82530092593</v>
       </c>
     </row>
@@ -2370,7 +2417,7 @@
       <c r="G85" s="6" t="n">
         <v>0.0081</v>
       </c>
-      <c r="H85" s="8" t="n">
+      <c r="H85" s="9" t="n">
         <v>46057.78736111111</v>
       </c>
     </row>
@@ -2396,7 +2443,7 @@
       <c r="G86" s="6" t="n">
         <v>0.0288</v>
       </c>
-      <c r="H86" s="8" t="n">
+      <c r="H86" s="9" t="n">
         <v>46087.69145833333</v>
       </c>
     </row>
@@ -2422,7 +2469,7 @@
       <c r="G87" s="6" t="n">
         <v>0.0276</v>
       </c>
-      <c r="H87" s="8" t="n">
+      <c r="H87" s="9" t="n">
         <v>46105.44788194444</v>
       </c>
     </row>
@@ -2448,7 +2495,7 @@
       <c r="G88" s="6" t="n">
         <v>0.0121</v>
       </c>
-      <c r="H88" s="8" t="n">
+      <c r="H88" s="9" t="n">
         <v>46199.24421296296</v>
       </c>
     </row>
@@ -2474,7 +2521,7 @@
       <c r="G89" s="6" t="n">
         <v>0.0128</v>
       </c>
-      <c r="H89" s="8" t="n">
+      <c r="H89" s="9" t="n">
         <v>46081.96149305555</v>
       </c>
     </row>
@@ -2500,7 +2547,7 @@
       <c r="G90" s="6" t="n">
         <v>0.0179</v>
       </c>
-      <c r="H90" s="8" t="n">
+      <c r="H90" s="9" t="n">
         <v>46105.66568287037</v>
       </c>
     </row>
@@ -2524,7 +2571,7 @@
       <c r="G91" s="6" t="n">
         <v>0.0089</v>
       </c>
-      <c r="H91" s="8" t="n">
+      <c r="H91" s="9" t="n">
         <v>46105.72203703703</v>
       </c>
     </row>
@@ -2550,7 +2597,7 @@
       <c r="G92" s="6" t="n">
         <v>0.0273</v>
       </c>
-      <c r="H92" s="8" t="n">
+      <c r="H92" s="9" t="n">
         <v>46124.13363425926</v>
       </c>
     </row>
@@ -2576,7 +2623,7 @@
       <c r="G93" s="6" t="n">
         <v>0.0246</v>
       </c>
-      <c r="H93" s="8" t="n">
+      <c r="H93" s="9" t="n">
         <v>46149.92591435185</v>
       </c>
     </row>
@@ -2602,7 +2649,7 @@
       <c r="G94" s="6" t="n">
         <v>0.018</v>
       </c>
-      <c r="H94" s="8" t="n">
+      <c r="H94" s="9" t="n">
         <v>46124.48695601852</v>
       </c>
     </row>
@@ -2628,7 +2675,7 @@
       <c r="G95" s="6" t="n">
         <v>0.0193</v>
       </c>
-      <c r="H95" s="8" t="n">
+      <c r="H95" s="9" t="n">
         <v>46206.7353125</v>
       </c>
     </row>
@@ -2654,7 +2701,7 @@
       <c r="G96" s="6" t="n">
         <v>0.0117</v>
       </c>
-      <c r="H96" s="8" t="n">
+      <c r="H96" s="9" t="n">
         <v>46145.62171296297</v>
       </c>
     </row>
@@ -2680,7 +2727,7 @@
       <c r="G97" s="6" t="n">
         <v>0.0072</v>
       </c>
-      <c r="H97" s="8" t="n">
+      <c r="H97" s="9" t="n">
         <v>46173.14605324074</v>
       </c>
     </row>
@@ -2706,7 +2753,7 @@
       <c r="G98" s="6" t="n">
         <v>0.0054</v>
       </c>
-      <c r="H98" s="8" t="n">
+      <c r="H98" s="9" t="n">
         <v>46145.58298611111</v>
       </c>
     </row>
@@ -2732,7 +2779,7 @@
       <c r="G99" s="6" t="n">
         <v>0.0246</v>
       </c>
-      <c r="H99" s="8" t="n">
+      <c r="H99" s="9" t="n">
         <v>46218.42115740741</v>
       </c>
     </row>
@@ -2758,7 +2805,7 @@
       <c r="G100" s="6" t="n">
         <v>0.0265</v>
       </c>
-      <c r="H100" s="8" t="n">
+      <c r="H100" s="9" t="n">
         <v>46162.66717592593</v>
       </c>
     </row>
@@ -2784,7 +2831,7 @@
       <c r="G101" s="6" t="n">
         <v>0.0036</v>
       </c>
-      <c r="H101" s="8" t="n">
+      <c r="H101" s="9" t="n">
         <v>46182.7936574074</v>
       </c>
     </row>
@@ -6875,7 +6922,7 @@
           <t>Seconds Played</t>
         </is>
       </c>
-      <c r="F399" s="2" t="inlineStr">
+      <c r="F399" s="8" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
@@ -6885,7 +6932,7 @@
           <t>Reaction</t>
         </is>
       </c>
-      <c r="H399" s="2" t="inlineStr">
+      <c r="H399" s="8" t="inlineStr">
         <is>
           <t>Royalty Amount</t>
         </is>
@@ -6898,7 +6945,7 @@
       <c r="B400" s="3" t="n">
         <v>4820</v>
       </c>
-      <c r="C400" s="8" t="n">
+      <c r="C400" s="9" t="n">
         <v>46160.09532407407</v>
       </c>
       <c r="D400" s="3" t="n">
@@ -6922,7 +6969,7 @@
       <c r="B401" s="3" t="n">
         <v>4821</v>
       </c>
-      <c r="C401" s="8" t="n">
+      <c r="C401" s="9" t="n">
         <v>46162.32160879629</v>
       </c>
       <c r="D401" s="3" t="n">
@@ -6946,7 +6993,7 @@
       <c r="B402" s="3" t="n">
         <v>4821</v>
       </c>
-      <c r="C402" s="8" t="n">
+      <c r="C402" s="9" t="n">
         <v>46163.89104166667</v>
       </c>
       <c r="D402" s="3" t="n"/>
@@ -6968,7 +7015,7 @@
       <c r="B403" s="3" t="n">
         <v>4821</v>
       </c>
-      <c r="C403" s="8" t="n">
+      <c r="C403" s="9" t="n">
         <v>46165.20553240741</v>
       </c>
       <c r="D403" s="3" t="n">
@@ -6996,7 +7043,7 @@
       <c r="B404" s="3" t="n">
         <v>4821</v>
       </c>
-      <c r="C404" s="8" t="n">
+      <c r="C404" s="9" t="n">
         <v>46166.09369212963</v>
       </c>
       <c r="D404" s="3" t="n">
@@ -7024,7 +7071,7 @@
       <c r="B405" s="3" t="n">
         <v>4827</v>
       </c>
-      <c r="C405" s="8" t="n">
+      <c r="C405" s="9" t="n">
         <v>46168.76226851852</v>
       </c>
       <c r="D405" s="3" t="n">
@@ -7048,7 +7095,7 @@
       <c r="B406" s="3" t="n">
         <v>4827</v>
       </c>
-      <c r="C406" s="8" t="n">
+      <c r="C406" s="9" t="n">
         <v>46172.02236111111</v>
       </c>
       <c r="D406" s="3" t="n"/>
@@ -7070,7 +7117,7 @@
       <c r="B407" s="3" t="n">
         <v>4827</v>
       </c>
-      <c r="C407" s="8" t="n">
+      <c r="C407" s="9" t="n">
         <v>46175.6665162037</v>
       </c>
       <c r="D407" s="3" t="n"/>
@@ -7096,7 +7143,7 @@
       <c r="B408" s="3" t="n">
         <v>4823</v>
       </c>
-      <c r="C408" s="8" t="n">
+      <c r="C408" s="9" t="n">
         <v>46177.8675</v>
       </c>
       <c r="D408" s="3" t="n"/>
@@ -7118,7 +7165,7 @@
       <c r="B409" s="3" t="n">
         <v>4818</v>
       </c>
-      <c r="C409" s="8" t="n">
+      <c r="C409" s="9" t="n">
         <v>46180.21228009259</v>
       </c>
       <c r="D409" s="3" t="n"/>
@@ -7140,7 +7187,7 @@
       <c r="B410" s="3" t="n">
         <v>4825</v>
       </c>
-      <c r="C410" s="8" t="n">
+      <c r="C410" s="9" t="n">
         <v>46186.41172453704</v>
       </c>
       <c r="D410" s="3" t="n">
@@ -7164,7 +7211,7 @@
       <c r="B411" s="3" t="n">
         <v>4823</v>
       </c>
-      <c r="C411" s="8" t="n">
+      <c r="C411" s="9" t="n">
         <v>46187.90158564815</v>
       </c>
       <c r="D411" s="3" t="n">
@@ -7192,7 +7239,7 @@
       <c r="B412" s="3" t="n">
         <v>4825</v>
       </c>
-      <c r="C412" s="8" t="n">
+      <c r="C412" s="9" t="n">
         <v>46188.03702546296</v>
       </c>
       <c r="D412" s="3" t="n">
@@ -7216,7 +7263,7 @@
       <c r="B413" s="3" t="n">
         <v>4825</v>
       </c>
-      <c r="C413" s="8" t="n">
+      <c r="C413" s="9" t="n">
         <v>46194.01096064815</v>
       </c>
       <c r="D413" s="3" t="n">
@@ -7244,7 +7291,7 @@
       <c r="B414" s="3" t="n">
         <v>4827</v>
       </c>
-      <c r="C414" s="8" t="n">
+      <c r="C414" s="9" t="n">
         <v>46199.69569444445</v>
       </c>
       <c r="D414" s="3" t="n"/>
@@ -7266,7 +7313,7 @@
       <c r="B415" s="3" t="n">
         <v>4829</v>
       </c>
-      <c r="C415" s="8" t="n">
+      <c r="C415" s="9" t="n">
         <v>46201.25351851852</v>
       </c>
       <c r="D415" s="3" t="n">
@@ -7290,7 +7337,7 @@
       <c r="B416" s="3" t="n">
         <v>4825</v>
       </c>
-      <c r="C416" s="8" t="n">
+      <c r="C416" s="9" t="n">
         <v>46202.31267361111</v>
       </c>
       <c r="D416" s="3" t="n">
@@ -7318,7 +7365,7 @@
       <c r="B417" s="3" t="n">
         <v>4825</v>
       </c>
-      <c r="C417" s="8" t="n">
+      <c r="C417" s="9" t="n">
         <v>46203.99975694445</v>
       </c>
       <c r="D417" s="3" t="n">
@@ -7346,7 +7393,7 @@
       <c r="B418" s="3" t="n">
         <v>4827</v>
       </c>
-      <c r="C418" s="8" t="n">
+      <c r="C418" s="9" t="n">
         <v>46210.49346064815</v>
       </c>
       <c r="D418" s="3" t="n"/>
@@ -7368,7 +7415,7 @@
       <c r="B419" s="3" t="n">
         <v>4824</v>
       </c>
-      <c r="C419" s="8" t="n">
+      <c r="C419" s="9" t="n">
         <v>46212.05660879629</v>
       </c>
       <c r="D419" s="3" t="n">
@@ -7396,7 +7443,7 @@
       <c r="B420" s="3" t="n">
         <v>4823</v>
       </c>
-      <c r="C420" s="8" t="n">
+      <c r="C420" s="9" t="n">
         <v>46223.97694444445</v>
       </c>
       <c r="D420" s="3" t="n">
@@ -7420,7 +7467,7 @@
       <c r="B421" s="3" t="n">
         <v>4828</v>
       </c>
-      <c r="C421" s="8" t="n">
+      <c r="C421" s="9" t="n">
         <v>46229.37763888889</v>
       </c>
       <c r="D421" s="3" t="n">
@@ -7444,7 +7491,7 @@
       <c r="B422" s="3" t="n">
         <v>4817</v>
       </c>
-      <c r="C422" s="8" t="n">
+      <c r="C422" s="9" t="n">
         <v>46236.90769675926</v>
       </c>
       <c r="D422" s="3" t="n">
@@ -7472,7 +7519,7 @@
       <c r="B423" s="3" t="n">
         <v>4826</v>
       </c>
-      <c r="C423" s="8" t="n">
+      <c r="C423" s="9" t="n">
         <v>46238.88868055555</v>
       </c>
       <c r="D423" s="3" t="n">
@@ -7496,7 +7543,7 @@
       <c r="B424" s="3" t="n">
         <v>4817</v>
       </c>
-      <c r="C424" s="8" t="n">
+      <c r="C424" s="9" t="n">
         <v>46239.76914351852</v>
       </c>
       <c r="D424" s="3" t="n">
@@ -7524,7 +7571,7 @@
       <c r="B425" s="3" t="n">
         <v>4817</v>
       </c>
-      <c r="C425" s="8" t="n">
+      <c r="C425" s="9" t="n">
         <v>46243.62960648148</v>
       </c>
       <c r="D425" s="3" t="n">
@@ -7552,7 +7599,7 @@
       <c r="B426" s="3" t="n">
         <v>4829</v>
       </c>
-      <c r="C426" s="8" t="n">
+      <c r="C426" s="9" t="n">
         <v>46253.56394675926</v>
       </c>
       <c r="D426" s="3" t="n">
@@ -7576,7 +7623,7 @@
       <c r="B427" s="3" t="n">
         <v>4817</v>
       </c>
-      <c r="C427" s="8" t="n">
+      <c r="C427" s="9" t="n">
         <v>46257.54693287037</v>
       </c>
       <c r="D427" s="3" t="n">
@@ -7600,7 +7647,7 @@
       <c r="B428" s="3" t="n">
         <v>4829</v>
       </c>
-      <c r="C428" s="8" t="n">
+      <c r="C428" s="9" t="n">
         <v>46259.98222222222</v>
       </c>
       <c r="D428" s="3" t="n"/>
@@ -7622,7 +7669,7 @@
       <c r="B429" s="3" t="n">
         <v>4817</v>
       </c>
-      <c r="C429" s="8" t="n">
+      <c r="C429" s="9" t="n">
         <v>46261.63834490741</v>
       </c>
       <c r="D429" s="3" t="n">
@@ -7650,7 +7697,7 @@
       <c r="B430" s="3" t="n">
         <v>4824</v>
       </c>
-      <c r="C430" s="8" t="n">
+      <c r="C430" s="9" t="n">
         <v>46263.2809837963</v>
       </c>
       <c r="D430" s="3" t="n"/>
@@ -7671,5 +7718,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>